<commit_message>
planillas intl: ec, cr y gt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/intl/cl/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/cl/sueldo-y-liquidacion-2026.xlsx
@@ -203,7 +203,7 @@
     <t>Último día de trabajo</t>
   </si>
   <si>
-    <t>Años completos</t>
+    <t>Antigüedad: años completos</t>
   </si>
   <si>
     <t>Última remuneración mensual</t>
@@ -212,7 +212,7 @@
     <t>Sueldo más lo fijo que recibes cada mes (colación, movilización, cotizaciones). Sin horas extra ni gratificación anual.</t>
   </si>
   <si>
-    <t>Última anualidad</t>
+    <t>Antigüedad: último aniversario</t>
   </si>
   <si>
     <t>Motivo del término</t>
@@ -221,7 +221,7 @@
     <t>Necesidades de la empresa (despido art. 161)</t>
   </si>
   <si>
-    <t>Meses desde la última anualidad</t>
+    <t>Antigüedad: meses</t>
   </si>
   <si>
     <t>Te avisaron con 30 días o más de anticipación</t>
@@ -230,7 +230,7 @@
     <t>No</t>
   </si>
   <si>
-    <t>Días sueltos</t>
+    <t>Antigüedad: días</t>
   </si>
   <si>
     <t>Días hábiles de vacaciones de años anteriores sin tomar</t>

</xml_diff>

<commit_message>
mundo: universales en el registro, cargadores en dos niveles, tabla del resultado y menú por grupos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/intl/cl/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/cl/sueldo-y-liquidacion-2026.xlsx
@@ -362,13 +362,13 @@
     <t>Unidad de Fomento (UF)</t>
   </si>
   <si>
-    <t>Valor al 9/10/2026</t>
+    <t>Valor al 13/10/2026</t>
   </si>
   <si>
     <t>CLP</t>
   </si>
   <si>
-    <t>9/10/2026</t>
+    <t>13/10/2026</t>
   </si>
   <si>
     <t>https://www.sii.cl/valores_y_fechas/uf/uf2026.htm</t>
@@ -2196,7 +2196,7 @@
         <v>115</v>
       </c>
       <c r="C11" s="35">
-        <v>41130.94</v>
+        <v>41152.13</v>
       </c>
       <c r="D11" s="34" t="s">
         <v>116</v>

</xml_diff>